<commit_message>
fix: align CS-real batch lookup with baseline fitting
</commit_message>
<xml_diff>
--- a/tutti-qc-assayprocess/Excel-data/103226061801&203226061801_260620.xlsx
+++ b/tutti-qc-assayprocess/Excel-data/103226061801&203226061801_260620.xlsx
@@ -786,7 +786,7 @@
       <c r="K2" s="36" t="n"/>
       <c r="L2" s="36" t="n"/>
       <c r="M2" s="36" t="n"/>
-      <c r="N2" s="35" t="n"/>
+      <c r="N2" s="35" t="inlineStr"/>
       <c r="O2" s="35" t="n"/>
       <c r="P2" s="36" t="n"/>
       <c r="Q2" s="36" t="n"/>
@@ -799,7 +799,11 @@
           <t>Product Code (REF)</t>
         </is>
       </c>
-      <c r="D3" s="36" t="n"/>
+      <c r="D3" s="36" t="inlineStr">
+        <is>
+          <t>905-115</t>
+        </is>
+      </c>
       <c r="E3" s="36" t="n"/>
       <c r="F3" s="36" t="n"/>
       <c r="G3" s="36" t="n"/>
@@ -834,7 +838,11 @@
       <c r="E4" s="36" t="n"/>
       <c r="F4" s="36" t="n"/>
       <c r="G4" s="36" t="n"/>
-      <c r="H4" s="35" t="n"/>
+      <c r="H4" s="35" t="inlineStr">
+        <is>
+          <t>1-000032-26061801</t>
+        </is>
+      </c>
       <c r="I4" s="35" t="n"/>
       <c r="J4" s="36" t="n"/>
       <c r="K4" s="36" t="n"/>
@@ -857,7 +865,11 @@
           <t>Device FW</t>
         </is>
       </c>
-      <c r="D5" s="36" t="n"/>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>Q1H250619013 / Q1H250619026 / Q1H260316001</t>
+        </is>
+      </c>
       <c r="E5" s="36" t="n"/>
       <c r="F5" s="36" t="n"/>
       <c r="G5" s="36" t="n"/>
@@ -867,7 +879,11 @@
       <c r="K5" s="36" t="n"/>
       <c r="L5" s="36" t="n"/>
       <c r="M5" s="36" t="n"/>
-      <c r="N5" s="35" t="n"/>
+      <c r="N5" s="35" t="inlineStr">
+        <is>
+          <t>14:41:00 / 14:42:43 / 14:56:07</t>
+        </is>
+      </c>
       <c r="O5" s="35" t="n"/>
       <c r="P5" s="36" t="n"/>
       <c r="Q5" s="36" t="n"/>
@@ -1068,15 +1084,31 @@
           <t>Beads Lot.</t>
         </is>
       </c>
-      <c r="D21" s="43" t="n"/>
+      <c r="D21" s="43" t="inlineStr">
+        <is>
+          <t>D:2312621X</t>
+        </is>
+      </c>
       <c r="E21" s="43" t="n"/>
-      <c r="F21" s="43" t="n"/>
+      <c r="F21" s="43" t="inlineStr">
+        <is>
+          <t>D:2572614Z</t>
+        </is>
+      </c>
       <c r="G21" s="43" t="n"/>
-      <c r="H21" s="43" t="n"/>
+      <c r="H21" s="43" t="inlineStr"/>
       <c r="I21" s="43" t="n"/>
-      <c r="J21" s="43" t="n"/>
+      <c r="J21" s="43" t="inlineStr">
+        <is>
+          <t>D:21926203</t>
+        </is>
+      </c>
       <c r="K21" s="43" t="n"/>
-      <c r="L21" s="43" t="n"/>
+      <c r="L21" s="43" t="inlineStr">
+        <is>
+          <t>D:10326207</t>
+        </is>
+      </c>
       <c r="M21" s="43" t="n"/>
       <c r="N21" s="43" t="n"/>
       <c r="O21" s="43" t="n"/>

</xml_diff>